<commit_message>
Updated UI and added email notification feature
</commit_message>
<xml_diff>
--- a/reports/risk_students.xlsx
+++ b/reports/risk_students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,20 +439,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>PERFORMANCE SCORE</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>RISK</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>REASON</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SUGGESTION</t>
         </is>
@@ -473,20 +478,25 @@
       <c r="D2" t="n">
         <v>89</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>gayee0131@gmail.com</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>78</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Attendance Risk</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Attendance below 75%</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Attend classes regularly.</t>
         </is>
@@ -507,20 +517,25 @@
       <c r="D3" t="n">
         <v>25</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>gayee0131@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>58.5</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Academic Risk</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Marks below 60</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Practice daily and revise important topics.</t>
         </is>
@@ -541,20 +556,25 @@
       <c r="D4" t="n">
         <v>89</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>gayee0131@gmail.com</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>61.5</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Attendance Risk</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Attendance below 75%</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Attend classes regularly.</t>
         </is>
@@ -575,20 +595,25 @@
       <c r="D5" t="n">
         <v>98</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>gayee0131@gmail.com</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>81.5</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Attendance Risk</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Attendance below 75%</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Attend classes regularly.</t>
         </is>
@@ -600,7 +625,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ajy</t>
+          <t>Ajay</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -609,20 +634,25 @@
       <c r="D6" t="n">
         <v>45</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>gayee0131@gmail.com</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>66</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Academic Risk</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Marks below 60</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Practice daily and revise important topics.</t>
         </is>

</xml_diff>

<commit_message>
Updated UI and improved email notification feature
</commit_message>
<xml_diff>
--- a/reports/risk_students.xlsx
+++ b/reports/risk_students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,25 +439,20 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PERFORMANCE SCORE</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>PERFORMANCE SCORE</t>
+          <t>RISK</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>RISK</t>
+          <t>REASON</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>REASON</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>SUGGESTION</t>
         </is>
@@ -465,40 +460,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arshad</t>
+          <t>Ravi</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D2" t="n">
-        <v>89</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>gayee0131@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>78</v>
+        <v>46</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Attendance Risk</t>
+          <t>Marks below 60</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Attendance below 75%</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Attend classes regularly.</t>
+          <t>Practice daily and revise important topics.</t>
         </is>
       </c>
     </row>
@@ -508,36 +498,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arjun</t>
+          <t>Nila</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>gayee0131@gmail.com</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>58.5</v>
+        <v>56</v>
+      </c>
+      <c r="E3" t="n">
+        <v>59</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Academic Risk</t>
+          <t>Low Attendance and Low Marks</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Marks below 60</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Practice daily and revise important topics.</t>
+          <t>Improve attendance and spend more time on academics.</t>
         </is>
       </c>
     </row>
@@ -547,114 +532,1085 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ayan</t>
+          <t>Nani</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="D4" t="n">
-        <v>89</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>gayee0131@gmail.com</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>61.5</v>
+        <v>52</v>
+      </c>
+      <c r="E4" t="n">
+        <v>60</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Attendance Risk</t>
+          <t>Low Attendance and Low Marks</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Attendance below 75%</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Attend classes regularly.</t>
+          <t>Improve attendance and spend more time on academics.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arun</t>
+          <t>Kiran</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D5" t="n">
-        <v>98</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>gayee0131@gmail.com</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>81.5</v>
+        <v>37</v>
+      </c>
+      <c r="E5" t="n">
+        <v>56</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Attendance Risk</t>
+          <t>Marks below 60</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Attendance below 75%</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Attend classes regularly.</t>
+          <t>Practice daily and revise important topics.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Arun</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>53</v>
+      </c>
+      <c r="D6" t="n">
+        <v>96</v>
+      </c>
+      <c r="E6" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>111</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Latha</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>44</v>
+      </c>
+      <c r="E7" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>112</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>67</v>
+      </c>
+      <c r="D8" t="n">
+        <v>39</v>
+      </c>
+      <c r="E8" t="n">
+        <v>53</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>113</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Naveen</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>114</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>87</v>
+      </c>
+      <c r="D10" t="n">
+        <v>29</v>
+      </c>
+      <c r="E10" t="n">
+        <v>58</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>115</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nikhil</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>65</v>
+      </c>
+      <c r="D11" t="n">
+        <v>47</v>
+      </c>
+      <c r="E11" t="n">
+        <v>56</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>117</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kavya</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>77</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>118</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nani</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>84</v>
+      </c>
+      <c r="D13" t="n">
+        <v>27</v>
+      </c>
+      <c r="E13" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>119</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Surya</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>66</v>
+      </c>
+      <c r="D14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E14" t="n">
+        <v>63</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>121</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Ajay</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>87</v>
-      </c>
-      <c r="D6" t="n">
-        <v>45</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>gayee0131@gmail.com</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>66</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="C15" t="n">
+        <v>64</v>
+      </c>
+      <c r="D15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E15" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>123</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Venu</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>64</v>
+      </c>
+      <c r="D16" t="n">
+        <v>82</v>
+      </c>
+      <c r="E16" t="n">
+        <v>73</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>124</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sita</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>58</v>
+      </c>
+      <c r="D17" t="n">
+        <v>47</v>
+      </c>
+      <c r="E17" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>125</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>64</v>
+      </c>
+      <c r="D18" t="n">
+        <v>37</v>
+      </c>
+      <c r="E18" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>126</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ajay</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>60</v>
+      </c>
+      <c r="D19" t="n">
+        <v>75</v>
+      </c>
+      <c r="E19" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>127</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pavi</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>59</v>
+      </c>
+      <c r="D20" t="n">
+        <v>80</v>
+      </c>
+      <c r="E20" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>128</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Deepa</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>67</v>
+      </c>
+      <c r="D21" t="n">
+        <v>83</v>
+      </c>
+      <c r="E21" t="n">
+        <v>75</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>129</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Surya</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>71</v>
+      </c>
+      <c r="D22" t="n">
+        <v>71</v>
+      </c>
+      <c r="E22" t="n">
+        <v>71</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>132</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Asha</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>62</v>
+      </c>
+      <c r="D23" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" t="n">
+        <v>51</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>133</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>83</v>
+      </c>
+      <c r="D24" t="n">
+        <v>38</v>
+      </c>
+      <c r="E24" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Academic Risk</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Marks below 60</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>135</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Pooja</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>75</v>
+      </c>
+      <c r="D25" t="n">
+        <v>27</v>
+      </c>
+      <c r="E25" t="n">
+        <v>51</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>136</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Raju</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>58</v>
+      </c>
+      <c r="D26" t="n">
+        <v>89</v>
+      </c>
+      <c r="E26" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>137</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ravi</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>91</v>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+      <c r="E27" t="n">
+        <v>61</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>138</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Teja</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>81</v>
+      </c>
+      <c r="D28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E28" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>139</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Riya</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>57</v>
+      </c>
+      <c r="D29" t="n">
+        <v>53</v>
+      </c>
+      <c r="E29" t="n">
+        <v>55</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>141</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Teja</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>96</v>
+      </c>
+      <c r="D30" t="n">
+        <v>48</v>
+      </c>
+      <c r="E30" t="n">
+        <v>72</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>142</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Venu</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>63</v>
+      </c>
+      <c r="D31" t="n">
+        <v>37</v>
+      </c>
+      <c r="E31" t="n">
+        <v>50</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>146</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Kavya</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>65</v>
+      </c>
+      <c r="D32" t="n">
+        <v>35</v>
+      </c>
+      <c r="E32" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Low Attendance and Low Marks</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Improve attendance and spend more time on academics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>147</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Asha</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>74</v>
+      </c>
+      <c r="D33" t="n">
+        <v>63</v>
+      </c>
+      <c r="E33" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>148</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Anu</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>98</v>
+      </c>
+      <c r="D34" t="n">
+        <v>53</v>
+      </c>
+      <c r="E34" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Academic Risk</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Marks below 60</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Practice daily and revise important topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>149</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Venu</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>63</v>
+      </c>
+      <c r="D35" t="n">
+        <v>86</v>
+      </c>
+      <c r="E35" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Attendance Risk</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Attendance below 75%</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Attend classes regularly.</t>
         </is>
       </c>
     </row>

</xml_diff>